<commit_message>
Ralph Lauren Boca: client-facing scrub and propose net 30.
Strip war-room diary (lock dates, rejected rates, leftover/template talk, anti-send meta) so the live page reads as a client exhibit. Keep set terms (21 weeks, $4,400/wk super, 10% CM, 1.5% insurance, 1% pre-con). Leave PM, CO markup, trades, and the grand total open. State LBC proposes net 30 against RL's net 90 policy, without the internal net 45 contrast. Align the CLIENT workbook payment and open-item notes.

Co-authored-by: lucasoffice <lucasoffice@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-03.xlsx
+++ b/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-03.xlsx
@@ -1019,7 +1019,7 @@
       </c>
       <c r="C13" s="78" t="inlineStr">
         <is>
-          <t>Ralph Lauren policy: net 90</t>
+          <t>LBC proposes net 30. Ralph Lauren stated policy: net 90.</t>
         </is>
       </c>
       <c r="D13" s="109" t="n"/>
@@ -1652,7 +1652,11 @@
         <f>H36*I36</f>
         <v/>
       </c>
-      <c r="K36" s="83" t="n"/>
+      <c r="K36" s="83" t="inlineStr">
+        <is>
+          <t>N/A — not used on this exhibit.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="B37" s="14" t="inlineStr">
@@ -1941,9 +1945,7 @@
           <t>Project Manager</t>
         </is>
       </c>
-      <c r="E48" s="17" t="n">
-        <v>3500</v>
-      </c>
+      <c r="E48" s="17"/>
       <c r="F48" s="20" t="inlineStr">
         <is>
           <t>Per Week</t>
@@ -1964,7 +1966,11 @@
         <f>E48*G48</f>
         <v/>
       </c>
-      <c r="K48" s="83" t="n"/>
+      <c r="K48" s="83" t="inlineStr">
+        <is>
+          <t>Open until a single figure is set.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="28" customHeight="1">
       <c r="B49" s="14" t="inlineStr">
@@ -2703,7 +2709,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="37" t="inlineStr">
         <is>
-          <t>Owner's representative: Charrette MG — Landis Kauffman, Claudia Mardones.  Payment: Ralph Lauren policy net 90.  Permit fees excluded / invoiced separately.  Sales tax invoiced separately.</t>
+          <t>Owner's representative: Charrette MG — Landis Kauffman, Claudia Mardones.  Payment: LBC proposes net 30 (Ralph Lauren stated policy is net 90).  Permit fees excluded / invoiced separately.  Sales tax invoiced separately.</t>
         </is>
       </c>
     </row>
@@ -2814,16 +2820,13 @@
     <row r="15">
       <c r="C15" s="40" t="inlineStr">
         <is>
-          <t>CO CM Fee % (follows project CM fee)</t>
-        </is>
-      </c>
-      <c r="E15" s="128">
-        <f>E12</f>
-        <v/>
-      </c>
+          <t>CO CM Fee % (open — separate from project CM fee)</t>
+        </is>
+      </c>
+      <c r="E15" s="128"/>
       <c r="G15" s="48" t="inlineStr">
         <is>
-          <t>Follows project CM fee.</t>
+          <t>Open — separate from the 10% project CM fee.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ralph Lauren Boca: deliverables hub, TBD costs, net 45 settlement band.
Hub links CLIENT xlsx (prefer 09-04 when present), cash-impact PDF filename, redline TBD, and #cody mount. Unknown costs read TBD. Opening ask stays net 30. Adds Jenny Morrow and Chris Deutschlaender. Cash PDF bytes not on this box — Cody drops the exact filename next to the xlsx.

Co-authored-by: lucasoffice <lucasoffice@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-03.xlsx
+++ b/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-03.xlsx
@@ -1019,7 +1019,7 @@
       </c>
       <c r="C13" s="78" t="inlineStr">
         <is>
-          <t>LBC proposes net 30. Ralph Lauren stated policy: net 90.</t>
+          <t>Opening ask: net 30. If net 30 is not accepted, net 45 is a possible settlement band. Ralph Lauren stated policy: net 90.</t>
         </is>
       </c>
       <c r="D13" s="109" t="n"/>
@@ -2709,7 +2709,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="37" t="inlineStr">
         <is>
-          <t>Owner's representative: Charrette MG — Landis Kauffman, Claudia Mardones.  Payment: LBC proposes net 30 (Ralph Lauren stated policy is net 90).  Permit fees excluded / invoiced separately.  Sales tax invoiced separately.</t>
+          <t>Owner's representative: Charrette MG — Landis Kauffman, Claudia Mardones.  Payment: opening ask net 30; net 45 is a possible settlement band if net 30 is not accepted (Ralph Lauren stated policy is net 90).  Permit fees excluded / invoiced separately.  Sales tax invoiced separately.</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2849,7 @@
     <row r="18">
       <c r="B18" s="42" t="inlineStr">
         <is>
-          <t>TRADE PACKAGES — amounts entered when bids are received</t>
+          <t>TRADE PACKAGES — TBD until bids are received (amounts stay blank for formula safety)</t>
         </is>
       </c>
     </row>
@@ -2879,9 +2879,7 @@
           <t>Trade package 1</t>
         </is>
       </c>
-      <c r="D20" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D20" s="52"/>
     </row>
     <row r="21">
       <c r="B21" s="53" t="n">
@@ -2892,9 +2890,7 @@
           <t>Trade package 2</t>
         </is>
       </c>
-      <c r="D21" s="55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D21" s="55"/>
     </row>
     <row r="22">
       <c r="B22" s="50" t="n">
@@ -2905,9 +2901,7 @@
           <t>Trade package 3</t>
         </is>
       </c>
-      <c r="D22" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D22" s="52"/>
     </row>
     <row r="23">
       <c r="B23" s="53" t="n">
@@ -2918,9 +2912,7 @@
           <t>Trade package 4</t>
         </is>
       </c>
-      <c r="D23" s="55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D23" s="55"/>
     </row>
     <row r="24">
       <c r="B24" s="50" t="n">
@@ -2931,9 +2923,7 @@
           <t>Trade package 5</t>
         </is>
       </c>
-      <c r="D24" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D24" s="52"/>
     </row>
     <row r="25">
       <c r="B25" s="53" t="n">
@@ -2944,9 +2934,7 @@
           <t>Trade package 6</t>
         </is>
       </c>
-      <c r="D25" s="55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D25" s="55"/>
     </row>
     <row r="26">
       <c r="B26" s="50" t="n">
@@ -2957,9 +2945,7 @@
           <t>Trade package 7</t>
         </is>
       </c>
-      <c r="D26" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D26" s="52"/>
     </row>
     <row r="27">
       <c r="B27" s="53" t="n">
@@ -2970,9 +2956,7 @@
           <t>Trade package 8</t>
         </is>
       </c>
-      <c r="D27" s="55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D27" s="55"/>
     </row>
     <row r="28">
       <c r="B28" s="50" t="n">
@@ -2983,9 +2967,7 @@
           <t>Trade package 9</t>
         </is>
       </c>
-      <c r="D28" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D28" s="52"/>
     </row>
     <row r="29">
       <c r="B29" s="53" t="n">
@@ -2996,9 +2978,7 @@
           <t>Trade package 10</t>
         </is>
       </c>
-      <c r="D29" s="55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D29" s="55"/>
     </row>
     <row r="30">
       <c r="B30" s="50" t="n">
@@ -3009,9 +2989,7 @@
           <t>Trade package 11</t>
         </is>
       </c>
-      <c r="D30" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D30" s="52"/>
     </row>
     <row r="31">
       <c r="B31" s="53" t="n">
@@ -3022,9 +3000,7 @@
           <t>Trade package 12</t>
         </is>
       </c>
-      <c r="D31" s="55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D31" s="55"/>
     </row>
     <row r="32">
       <c r="B32" s="50" t="n">
@@ -3035,9 +3011,7 @@
           <t>Trade package 13</t>
         </is>
       </c>
-      <c r="D32" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D32" s="52"/>
     </row>
     <row r="33">
       <c r="B33" s="53" t="n">
@@ -3048,9 +3022,7 @@
           <t>Trade package 14</t>
         </is>
       </c>
-      <c r="D33" s="55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D33" s="55"/>
     </row>
     <row r="34">
       <c r="B34" s="50" t="n">
@@ -3061,9 +3033,7 @@
           <t>Trade package 15</t>
         </is>
       </c>
-      <c r="D34" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D34" s="52"/>
     </row>
     <row r="35">
       <c r="B35" s="53" t="n">
@@ -3074,9 +3044,7 @@
           <t>Trade package 16</t>
         </is>
       </c>
-      <c r="D35" s="55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D35" s="55"/>
     </row>
     <row r="36">
       <c r="B36" s="50" t="n">
@@ -3087,9 +3055,7 @@
           <t>Trade package 17</t>
         </is>
       </c>
-      <c r="D36" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D36" s="52"/>
     </row>
     <row r="37">
       <c r="B37" s="53" t="n">
@@ -3100,9 +3066,7 @@
           <t>Trade package 18</t>
         </is>
       </c>
-      <c r="D37" s="55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D37" s="55"/>
     </row>
     <row r="38">
       <c r="B38" s="50" t="n">
@@ -3113,9 +3077,7 @@
           <t>Trade package 19</t>
         </is>
       </c>
-      <c r="D38" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D38" s="52"/>
     </row>
     <row r="39">
       <c r="B39" s="53" t="n">
@@ -3126,9 +3088,7 @@
           <t>Trade package 20</t>
         </is>
       </c>
-      <c r="D39" s="55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D39" s="55"/>
     </row>
     <row r="40">
       <c r="C40" s="56" t="inlineStr">
@@ -3190,7 +3150,7 @@
       </c>
       <c r="G44" s="83" t="inlineStr">
         <is>
-          <t>Entered commercial terms. Trade-package rows are $0 until bids are received.</t>
+          <t>Entered commercial terms. Trade-package rows are TBD until bids are received. Blank amounts do not invent a job total.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ralph Lauren Boca: lock PM $3,500/wk + 4 trips and 5-month parking.
Shawn Rasmusen is Estimating / Project Manager. Parking is 5 months × $250 = $1,250 from the 21-week duration. Trades, sprinkler-shutdown count, CO markup, and grand total stay Open / TBD.

Co-authored-by: lucasoffice <lucasoffice@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-03.xlsx
+++ b/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-03.xlsx
@@ -930,7 +930,7 @@
     <row r="5" ht="36" customHeight="1">
       <c r="B5" s="30" t="inlineStr">
         <is>
-          <t>Commercial terms: 21 weeks · $4,400/wk superintendent · 10% CM fee · 1.5% liability insurance · 1% pre-construction, payable with first pay application / NTP.</t>
+          <t>Commercial terms: 21 weeks · $4,400/wk superintendent · $3,500/wk project manager (Shawn Rasmusen) + 4 trips · 5 months parking × $250 = $1,250 · 10% CM fee · 1.5% liability insurance · 1% pre-construction, payable with first pay application / NTP.</t>
         </is>
       </c>
     </row>
@@ -1945,13 +1945,17 @@
           <t>Project Manager</t>
         </is>
       </c>
-      <c r="E48" s="17"/>
+      <c r="E48" s="17" t="n">
+        <v>3500</v>
+      </c>
       <c r="F48" s="20" t="inlineStr">
         <is>
           <t>Per Week</t>
         </is>
       </c>
-      <c r="G48" s="39" t="n"/>
+      <c r="G48" s="39" t="n">
+        <v>21</v>
+      </c>
       <c r="H48" s="20" t="inlineStr">
         <is>
           <t>Weeks</t>
@@ -1968,7 +1972,7 @@
       </c>
       <c r="K48" s="83" t="inlineStr">
         <is>
-          <t>Open until a single figure is set.</t>
+          <t>Shawn Rasmusen. $3,500 per week × 21 weeks + 4 trips.</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2787,7 @@
       </c>
       <c r="G11" s="83" t="inlineStr">
         <is>
-          <t>$4,400 per week superintendent.</t>
+          <t>$4,400 per week superintendent. Project manager $3,500/wk (Shawn Rasmusen) + 4 trips — see GC bid form C-5.</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3161,7 @@
     <row r="46" ht="20" customHeight="1">
       <c r="B46" s="60" t="inlineStr">
         <is>
-          <t>Cost-plus CM fee form. Duration 21 weeks. Superintendent $4,400/wk. CM fee 10%. Insurance 1.5%. Pre-construction 1% of project total, payable with first pay application / NTP.</t>
+          <t>Cost-plus CM fee form. Duration 21 weeks. Superintendent $4,400/wk. Project manager $3,500/wk + 4 trips. Parking 5 months × $250 = $1,250. CM fee 10%. Insurance 1.5%. Pre-construction 1% of project total, payable with first pay application / NTP.</t>
         </is>
       </c>
     </row>
@@ -3385,19 +3389,21 @@
           <t>$/month</t>
         </is>
       </c>
-      <c r="E10" s="99" t="n"/>
+      <c r="E10" s="99" t="n">
+        <v>5</v>
+      </c>
       <c r="F10" s="95">
         <f>IF(E10="","",C10*E10)</f>
         <v/>
       </c>
       <c r="G10" s="90" t="inlineStr">
         <is>
-          <t>Qty pending</t>
+          <t>Set — 5 months</t>
         </is>
       </c>
       <c r="H10" s="97" t="inlineStr">
         <is>
-          <t>$250 per month. Month count to be confirmed.</t>
+          <t>$250 × 5 months = $1,250 (from 21-week duration).</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3506,7 @@
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="103" t="inlineStr">
         <is>
-          <t>Parking months and sprinkler-shutdown count to be confirmed. Permit fees and sales tax invoiced separately.</t>
+          <t>Parking is set at 5 months × $250 = $1,250. Sprinkler-shutdown count still Open / TBD. Permit fees and sales tax invoiced separately.</t>
         </is>
       </c>
     </row>

</xml_diff>